<commit_message>
Use Cambium22 for solar thermal, the latest year in which Cambium builds solar thermal during the mid case model run
</commit_message>
<xml_diff>
--- a/InputData/elec/ELCCAfR/ELCCAfR Effective Load Carrying Capability Adjustment for Reliability.xlsx
+++ b/InputData/elec/ELCCAfR/ELCCAfR Effective Load Carrying Capability Adjustment for Reliability.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Hourly VRE Capacity Factors at Pinned Peak Days (solar PV, solar thermal, onshore wind)</t>
+          <t>Hourly VRE Capacity Factors at Pinned Peak Days (solar PV, onshore wind)</t>
         </is>
       </c>
       <c r="C3" s="10" t="n"/>
@@ -602,7 +602,7 @@
       <c r="A8" s="10" t="n"/>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>MidCase scenario, weather year 2012, USA national resolution, hourly (Eastern Time in the source file), 2025 model year. File: Cambium24_MidCase_hourly_usa_2025.csv. The hourly file is not pasted into this workbook - see the No raw source tabs note below. Manipulation: per-tech hourly output is read at each hour-of-day on the pinned Summer Peak and Winter Peak days (see pinned-day source below), and each output cell is computed as 70%-exceedance output / mean output across those days at that hour-of-day. Nameplate capacity cancels out of the ratio, so hourly generation (MWh) is used directly in place of capacity factors. Moved from Cambium 2022 to Cambium 2024 on 2026-08-26 (Megan): the national model now uses Cambium24, which also matches the vintage of the SHELF clustering that supplies the pinned days. STATE models stay on Cambium 2022, which retains state disaggregation that Cambium24 does not provide - so this national file is no longer interchangeable with the state ELCCAfR files (see Deployment).</t>
+          <t>MidCase scenario, weather year 2012, USA national resolution, hourly (Eastern Time in the source file), 2025 model year. File: Cambium24_MidCase_hourly_usa_2025.csv. Applies to solar PV and onshore wind; offshore wind and solar thermal take different sources (see the next block). The hourly file is not pasted into this workbook - see the No raw source tabs note below. Manipulation: per-tech hourly output is read at each hour-of-day on the pinned Summer Peak and Winter Peak days (see pinned-day source below), and each output cell is computed as 70%-exceedance output / mean output across those days at that hour-of-day. Nameplate capacity cancels out of the ratio, so hourly generation (MWh) is used directly in place of capacity factors. Moved from Cambium 2022 to Cambium 2024 on 2026-08-26 (Megan): the national model now uses Cambium24, which also matches the vintage of the SHELF clustering that supplies the pinned days. STATE models stay on Cambium 2022, which retains state disaggregation Cambium24 does not provide - so this national file is no longer interchangeable with the state ELCCAfR files (see Deployment).</t>
         </is>
       </c>
       <c r="C8" s="10" t="n"/>
@@ -620,7 +620,7 @@
       <c r="A10" s="10" t="n"/>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Hourly Offshore Wind Capacity Factors - 2040 model year (offshore wind tab only)</t>
+          <t>Exceptions - offshore wind (later model year) and solar thermal (Cambium 2022)</t>
         </is>
       </c>
       <c r="C10" s="10" t="n"/>
@@ -642,7 +642,7 @@
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>NREL Cambium Scenarios 2024</t>
+          <t>NREL Cambium Scenarios 2024 (offshore wind) / 2022 (solar thermal)</t>
         </is>
       </c>
       <c r="C12" s="10" t="n"/>
@@ -653,7 +653,7 @@
       <c r="A13" s="10" t="n"/>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 / 2022</t>
         </is>
       </c>
       <c r="C13" s="10" t="n"/>
@@ -675,7 +675,7 @@
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Same file family and method as above, but the 2040 model year (Cambium24_MidCase_hourly_usa_2040.csv, ~50 GW national offshore fleet). A later model year is required because the near-term offshore fleet is too small for the statistic to describe resource behaviour rather than single-site weather: the Cambium24 2025 offshore fleet is 1.7 GW, versus 50.3 GW in 2040. Every Cambium model year shares the 2012 weather year, so the pinned peak days line up across model years and the method is otherwise unchanged. Solar thermal has no equivalent option - Cambium24 builds essentially no CSP in any model year (zero generating hours in 2025; a 61 MW stub in 2040) - so every solar thermal cell falls to the degenerate 1.0 case. That is immaterial in the national model, where BHRaSYC-StartYearCapacities gives solar thermal zero capacity.</t>
+          <t>OFFSHORE WIND: same file family and method as above, but the 2040 model year (Cambium24_MidCase_hourly_usa_2040.csv, ~50 GW national offshore fleet). A later model year is required because the near-term offshore fleet is too small for the statistic to describe resource behaviour rather than single-site weather: the Cambium24 2025 offshore fleet is 1.7 GW, versus 50.3 GW in 2040. Every Cambium model year shares the 2012 weather year, so the pinned peak days line up across model years and the method is otherwise unchanged. SOLAR THERMAL: computed from Cambium22_MidCase_hourly_usa_2024.csv, because Cambium24 has no usable CSP fleet in any model year or scenario - 59 MW in MidCase (zero generating hours in 2025), 163 MW in the most CSP-heavy Cambium24 scenario, and zero in Cambium23 - whereas Cambium22 carries 1,323 MW across CA (918), AZ (296) and NV (110), flat from 2024 through 2040. The statistic, pinned days and degenerate/cap rules are identical to the other techs; only the source vintage differs. Solar thermal is immaterial in the national model regardless: BHRaSYC-StartYearCapacities gives it zero capacity.</t>
         </is>
       </c>
       <c r="C15" s="10" t="n"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Per (tech, slice, hour) cell: ELCCAfR = 70%-exceedance CF / mean CF across the pinned peak days at that hour-of-day (70% exceedance = the 30th percentile of the pinned-day sample, linearly interpolated), with both statistics taken at the same hour-of-day. Adopted 2026-08-26, replacing a minimum-CF numerator: the minimum over 10-11 pinned days is a ~96% exceedance standard that no adopted accreditation framework uses, and one calm day sets the credit. The 70% exceedance level follows the CPUC Slice-of-Day resource-adequacy framework (D.23-04-010, levels updated triennially per D.24-06-004), which sets hourly wind and solar qualifying capacity from 70%-exceedance profiles over peak load days; expectation-based ELCC (PJM marginal ELCC, the NREL capacity-value literature) sits higher still, at the mean. Verify the exact exceedance language against D.23-04-010 and the current RA filing guide before any external use. Degenerate cells (negligible mean CF, e.g. solar overnight) are 1.0 - no effect, since SYSHECF is ~0 there anyway. Cells are capped at 1.0: unlike min/mean, a percentile numerator can exceed the mean where the pinned-day sample is left-skewed, and ELCCAfR is a derate, never a bonus. Three cells cap under the current data, all in offshore wind Winter Peak. Solar PV, solar thermal and onshore wind use the Cambium 2025 model year; offshore wind uses 2040 (see Sources).</t>
+          <t>Per (tech, slice, hour) cell: ELCCAfR = 70%-exceedance CF / mean CF across the pinned peak days at that hour-of-day (70% exceedance = the 30th percentile of the pinned-day sample, linearly interpolated), with both statistics taken at the same hour-of-day. Adopted 2026-08-26, replacing a minimum-CF numerator: the minimum over 10-11 pinned days is a ~96% exceedance standard that no adopted accreditation framework uses, and one calm day sets the credit. The 70% exceedance level follows the CPUC Slice-of-Day resource-adequacy framework (D.23-04-010, levels updated triennially per D.24-06-004), which sets hourly wind and solar qualifying capacity from 70%-exceedance profiles over peak load days; expectation-based ELCC (PJM marginal ELCC, the NREL capacity-value literature) sits higher still, at the mean. Verify the exact exceedance language against D.23-04-010 and the current RA filing guide before any external use. Degenerate cells (negligible mean CF, e.g. solar overnight) are 1.0 - no effect, since SYSHECF is ~0 there anyway. Cells are capped at 1.0: unlike min/mean, a percentile numerator can exceed the mean where the pinned-day sample is left-skewed, and ELCCAfR is a derate, never a bonus. Under the current data 14 cells cap - 3 in offshore wind Winter Peak and 11 in solar thermal, whose three-site fleet is the most skewed sample. Two cells are exactly zero (solar thermal shoulder hours), meaning at least 30% of pinned days had no output at that hour; the previously deployed min-based file had a zero in the same summer hour. Model years: solar PV and onshore wind Cambium24 2025; offshore wind Cambium24 2040; solar thermal Cambium22 2024 (see Sources).</t>
         </is>
       </c>
       <c r="C31" s="10" t="n"/>
@@ -877,7 +877,7 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Unlike most EPS input workbooks, the raw Cambium hourly files (8,760 rows x ~78 columns per model year) are not pasted into source tabs here, and the output tabs hold values rather than formulas. The national values in this workbook are produced by recompute_elccafr_national.py, which reads the pinned day-of-year to timeslice assignment from the pasted Cambium hourly source tab of the deployed SHELF workbook and verifies on every run that reading the Cambium24 2025 CSV reproduces that tab cell-for-cell (48/48 cells per tech) before writing anything. Note that the state-data-pipeline ELCCAfR builder no longer reproduces these national values, because the national file moved to Cambium24 while the builder and the state files remain on Cambium22. The per-state workbooks carry pasted pinned-day source tabs and live MIN/AVERAGE formulas - see any state ELCCAfR workbook in state-eps-data-repository for the fully auditable state version of this calculation.</t>
+          <t>Unlike most EPS input workbooks, the raw Cambium hourly files (8,760 rows x ~78 columns per model year) are not pasted into source tabs here, and the output tabs hold values rather than formulas. The national values in this workbook are produced by recompute_elccafr_national.py, which reads the pinned day-of-year to timeslice assignment from the pasted Cambium hourly source tab of the deployed SHELF workbook and verifies on every run that reading the Cambium24 2025 CSV reproduces that tab cell-for-cell (48/48 cells per tech) before writing anything. Note that the state-data-pipeline ELCCAfR builder no longer reproduces these national values, because the national file moved to Cambium24 while the builder and the state files remain on Cambium22. Note also that the PREVIOUSLY deployed national values could not be reproduced from any pinned-day set available in this repo: they were computed against a 27-summer / 20-winter-peak-day clustering (the day counts carried by commit 5243d9fe, which introduced them), while the deployed SHELF has carried 11 / 10 since commit 6fdfe6dd two days later - so the old values were stale with respect to the pinned days they claimed. The current values are computed on the deployed pinned days and gated against them. The per-state workbooks carry pasted pinned-day source tabs and live MIN/AVERAGE formulas - see any state ELCCAfR workbook in state-eps-data-repository for the fully auditable state version.</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -892,7 +892,7 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>CHANGED 2026-08-26: this national file is NO LONGER byte-identical to the state ELCCAfR files and must not be synced over them. National uses Cambium24; state models stay on Cambium22, which retains the state disaggregation Cambium24 does not provide (Megan, 2026-08-26). Previously all 50 state ELCCAfR-offshore-wind.csv files inherited this file unchanged (state-eps-data-repository commit 08659643df). Any model-sync step that copies the national ELCCAfR folder into state input trees needs to be updated to exclude it, or states will silently pick up the Cambium24 national values. The state files also still carry the min/mean statistic; converting them to 70% exceedance on their Cambium22 basis is separate work.</t>
+          <t>CHANGED 2026-08-26: this national file is NO LONGER byte-identical to the state ELCCAfR files and must not be synced over them. National uses Cambium24 (except solar thermal, on Cambium22 for lack of a Cambium24 CSP fleet); state models stay on Cambium22, which retains the state disaggregation Cambium24 does not provide (Megan, 2026-08-26). Previously all 50 state ELCCAfR-offshore-wind.csv files inherited this file unchanged (state-eps-data-repository commit 08659643df). Any model-sync step that copies the national ELCCAfR folder into state input trees needs to be updated to exclude it, or states will silently pick up the Cambium24 national values. The state files also still carry the min/mean statistic; converting them to 70% exceedance on their Cambium22 basis is separate work.</t>
         </is>
       </c>
       <c r="C34" s="10" t="n"/>
@@ -12707,10 +12707,10 @@
         <v>1</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>1</v>
+        <v>0.8639</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>1</v>
@@ -12719,10 +12719,10 @@
         <v>1</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>1</v>
+        <v>0.9716</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>1</v>
+        <v>0.9671999999999999</v>
       </c>
       <c r="O6" s="7" t="n">
         <v>1</v>
@@ -12743,10 +12743,10 @@
         <v>1</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>1</v>
+        <v>0.9313</v>
       </c>
       <c r="V6" s="7" t="n">
-        <v>1</v>
+        <v>0.7022</v>
       </c>
       <c r="W6" s="5" t="n">
         <v>1</v>
@@ -12792,22 +12792,22 @@
         <v>1</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1</v>
+        <v>0.2419</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1</v>
+        <v>0.9532</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>1</v>
+        <v>0.8804</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>1</v>
+        <v>0.9782</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>1</v>
+        <v>0.9895</v>
       </c>
       <c r="P7" s="7" t="n">
-        <v>1</v>
+        <v>0.9927</v>
       </c>
       <c r="Q7" s="7" t="n">
         <v>1</v>
@@ -12819,10 +12819,10 @@
         <v>1</v>
       </c>
       <c r="T7" s="7" t="n">
-        <v>1</v>
+        <v>0.8902</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V7" s="5" t="n">
         <v>1</v>

</xml_diff>